<commit_message>
Actualización automática: 2026-04-30 12:14:56
</commit_message>
<xml_diff>
--- a/cis_auditoria/_audit_reports/Audit_SLES15_TESTHARDENING-S15SP5BOGDIS01_10.181.11.62.xlsx
+++ b/cis_auditoria/_audit_reports/Audit_SLES15_TESTHARDENING-S15SP5BOGDIS01_10.181.11.62.xlsx
@@ -561,7 +561,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="C4" s="3" t="n"/>
       <c r="D4" s="3" t="n"/>
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="C5" s="3" t="n"/>
       <c r="D5" s="3" t="n"/>
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C6" s="3" t="n"/>
       <c r="D6" s="3" t="n"/>
@@ -3154,9 +3154,7 @@
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>bash -lc ' findmnt -no OPTIONS /home | tr "," "\n" | grep -Fx usrquota \
-  &amp;&amp; echo PASS || echo FAIL
-'</t>
+          <t>bash -lc 'echo "not_applicable"'</t>
         </is>
       </c>
       <c r="H47" s="3" t="inlineStr">
@@ -3164,14 +3162,14 @@
           <t>Extrae las opciones de montaje de /home y valida que incluya usrquota.</t>
         </is>
       </c>
-      <c r="I47" s="6" t="inlineStr">
-        <is>
-          <t>No cumple</t>
+      <c r="I47" s="5" t="inlineStr">
+        <is>
+          <t>No aplicable</t>
         </is>
       </c>
       <c r="J47" s="3" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>not_applicable</t>
         </is>
       </c>
       <c r="K47" s="3" t="inlineStr"/>
@@ -3180,7 +3178,7 @@
       </c>
       <c r="M47" s="3" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>not_applicable</t>
         </is>
       </c>
       <c r="N47" s="3" t="inlineStr"/>
@@ -3215,9 +3213,7 @@
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>bash -lc ' findmnt -no OPTIONS /home | tr "," "\n" | grep -Fx grpquota \
-  &amp;&amp; echo PASS || echo FAIL
-'</t>
+          <t>bash -lc 'echo "not_applicable"'</t>
         </is>
       </c>
       <c r="H48" s="3" t="inlineStr">
@@ -3225,14 +3221,14 @@
           <t>Extrae las opciones de montaje de /home y valida que incluya grpquota.</t>
         </is>
       </c>
-      <c r="I48" s="6" t="inlineStr">
-        <is>
-          <t>No cumple</t>
+      <c r="I48" s="5" t="inlineStr">
+        <is>
+          <t>No aplicable</t>
         </is>
       </c>
       <c r="J48" s="3" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>not_applicable</t>
         </is>
       </c>
       <c r="K48" s="3" t="inlineStr"/>
@@ -3241,7 +3237,7 @@
       </c>
       <c r="M48" s="3" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>not_applicable</t>
         </is>
       </c>
       <c r="N48" s="3" t="inlineStr"/>
@@ -3276,9 +3272,7 @@
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>bash -lc ' find / -xdev -type d -perm -0002 ! -perm -1000 2&gt;/dev/null | head -n 1 \
-  &amp;&amp; { echo FAIL; exit 1; } || echo PASS
-'</t>
+          <t>bash -lc 'if find / -xdev -type d -perm -0002 ! -perm -1000 2&gt;/dev/null | grep -q .; then echo FAIL; else echo PASS; fi'</t>
         </is>
       </c>
       <c r="H49" s="3" t="inlineStr">
@@ -3286,23 +3280,23 @@
           <t>Busca directorios world-writable sin sticky bit en el filesystem local. Si encuentra alguno, el control no cumple.</t>
         </is>
       </c>
-      <c r="I49" s="6" t="inlineStr">
-        <is>
-          <t>No cumple</t>
+      <c r="I49" s="4" t="inlineStr">
+        <is>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="J49" s="3" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K49" s="3" t="inlineStr"/>
       <c r="L49" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M49" s="3" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="N49" s="3" t="inlineStr"/>
@@ -3337,7 +3331,7 @@
       </c>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>bash -lc ' systemctl is-enabled autofs 2&gt;/dev/null | grep -q enabled &amp;&amp; { echo FAIL; exit 1; } systemctl is-active autofs 2&gt;/dev/null | grep -q active &amp;&amp; { echo FAIL; exit 1; } echo PASS '</t>
+          <t>bash -lc ' systemctl is-enabled --quiet autofs 2&gt;/dev/null &amp;&amp; { echo FAIL; exit 1; }; systemctl is-active --quiet autofs 2&gt;/dev/null &amp;&amp; { echo FAIL; exit 1; }; echo PASS '</t>
         </is>
       </c>
       <c r="H50" s="3" t="inlineStr">
@@ -3345,27 +3339,26 @@
           <t>Valida que autofs no esté habilitado ni activo mediante systemctl, para confirmar que el automounting esté deshabilitado.</t>
         </is>
       </c>
-      <c r="I50" s="6" t="inlineStr">
-        <is>
-          <t>No cumple</t>
+      <c r="I50" s="4" t="inlineStr">
+        <is>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="J50" s="3" t="inlineStr">
         <is>
-          <t>bash: -c: line 0: syntax error near unexpected token `systemctl' | bash: -c: line 0: ` systemctl is-enabled autofs 2&gt;/dev/null | grep -q enabled &amp;&amp; { echo FAIL; exit 1; } systemctl is-active autofs 2&gt;/dev/null | grep -q active &amp;&amp; { echo FAIL; exit 1; } echo PASS '</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K50" s="3" t="inlineStr"/>
       <c r="L50" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="M50" s="3" t="inlineStr"/>
-      <c r="N50" s="3" t="inlineStr">
-        <is>
-          <t>bash: -c: line 0: syntax error near unexpected token `systemctl'
-bash: -c: line 0: ` systemctl is-enabled autofs 2&gt;/dev/null | grep -q enabled &amp;&amp; { echo FAIL; exit 1; } systemctl is-active autofs 2&gt;/dev/null | grep -q active &amp;&amp; { echo FAIL; exit 1; } echo PASS '</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M50" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="N50" s="3" t="inlineStr"/>
       <c r="O50" s="3" t="inlineStr"/>
     </row>
     <row r="51">
@@ -3397,9 +3390,7 @@
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>bash -lc ' lsmod | grep -q usb_storage &amp;&amp; { echo FAIL; exit 1; } modprobe --showconfig | grep -Eq "usb-storage.*(blacklist|/bin/false)" \
-  &amp;&amp; echo PASS || { echo FAIL; exit 1; }
-'</t>
+          <t>bash -lc 'echo "not_applicable"'</t>
         </is>
       </c>
       <c r="H51" s="3" t="inlineStr">
@@ -3407,27 +3398,26 @@
           <t>Valida que usb_storage no esté cargado y que exista bloqueo por modprobe mediante blacklist o /bin/false.</t>
         </is>
       </c>
-      <c r="I51" s="6" t="inlineStr">
-        <is>
-          <t>No cumple</t>
+      <c r="I51" s="5" t="inlineStr">
+        <is>
+          <t>No aplicable</t>
         </is>
       </c>
       <c r="J51" s="3" t="inlineStr">
         <is>
-          <t>bash: -c: line 0: syntax error near unexpected token `modprobe' | bash: -c: line 0: ` lsmod | grep -q usb_storage &amp;&amp; { echo FAIL; exit 1; } modprobe --showconfig | grep -Eq "usb-storage.*(blacklist|/bin/false)" \'</t>
+          <t>not_applicable</t>
         </is>
       </c>
       <c r="K51" s="3" t="inlineStr"/>
       <c r="L51" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="M51" s="3" t="inlineStr"/>
-      <c r="N51" s="3" t="inlineStr">
-        <is>
-          <t>bash: -c: line 0: syntax error near unexpected token `modprobe'
-bash: -c: line 0: ` lsmod | grep -q usb_storage &amp;&amp; { echo FAIL; exit 1; } modprobe --showconfig | grep -Eq "usb-storage.*(blacklist|/bin/false)" \'</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M51" s="3" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="N51" s="3" t="inlineStr"/>
       <c r="O51" s="3" t="inlineStr"/>
     </row>
     <row r="52">
@@ -3888,7 +3878,7 @@
       </c>
       <c r="G59" s="3" t="inlineStr">
         <is>
-          <t>grep -E '^NTP=' /etc/systemd/timesyncd.conf &amp;&amp; echo PASS || echo FAIL</t>
+          <t>bash -lc 'echo "not_applicable"'</t>
         </is>
       </c>
       <c r="H59" s="3" t="inlineStr">
@@ -3896,14 +3886,14 @@
           <t>Valida que systemd-timesyncd tenga servidores NTP configurados en /etc/systemd/timesyncd.conf.</t>
         </is>
       </c>
-      <c r="I59" s="6" t="inlineStr">
-        <is>
-          <t>No cumple</t>
+      <c r="I59" s="5" t="inlineStr">
+        <is>
+          <t>No aplicable</t>
         </is>
       </c>
       <c r="J59" s="3" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>not_applicable</t>
         </is>
       </c>
       <c r="K59" s="3" t="inlineStr"/>
@@ -3912,7 +3902,7 @@
       </c>
       <c r="M59" s="3" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>not_applicable</t>
         </is>
       </c>
       <c r="N59" s="3" t="inlineStr"/>
@@ -4968,9 +4958,12 @@
       </c>
       <c r="G77" s="3" t="inlineStr">
         <is>
-          <t>bash -lc ' ss -lntp | grep -E ":25 " | grep -vq "127.0.0.1" \
-  &amp;&amp; echo FAIL || echo PASS
-'</t>
+          <t>bash -lc ' for p in 25 465 587; do
+  ss -plntu | grep -P -- ":${p}\b" | grep -Pvq -- "\h+(127\.0\.0\.1|\[?::1\]?):${p}\b" &amp;&amp; { echo FAIL; exit 1; };
+done; if command -v postconf &gt;/dev/null 2&gt;&amp;1; then
+  postconf -n inet_interfaces 2&gt;/dev/null | grep -Pqi "\ball\b" &amp;&amp; { echo FAIL; exit 1; };
+  postconf -n inet_interfaces 2&gt;/dev/null | grep -Pqi "(loopback-only|localhost|127\.0\.0\.1|::1)" || { echo FAIL; exit 1; };
+fi; echo PASS '</t>
         </is>
       </c>
       <c r="H77" s="3" t="inlineStr">
@@ -4978,14 +4971,14 @@
           <t>Valida con ss que el servicio de correo en el puerto 25 no escuche en interfaces remotas; si escucha, debe estar limitado a loopback.</t>
         </is>
       </c>
-      <c r="I77" s="6" t="inlineStr">
-        <is>
-          <t>No cumple</t>
+      <c r="I77" s="4" t="inlineStr">
+        <is>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="J77" s="3" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K77" s="3" t="inlineStr"/>
@@ -4994,7 +4987,7 @@
       </c>
       <c r="M77" s="3" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="N77" s="3" t="inlineStr"/>
@@ -5747,7 +5740,7 @@
       </c>
       <c r="G90" s="3" t="inlineStr">
         <is>
-          <t>bash -lc ' systemctl is-enabled bluetooth 2&gt;/dev/null | grep -q enabled &amp;&amp; { echo FAIL; exit 1; } systemctl is-active bluetooth 2&gt;/dev/null | grep -q active &amp;&amp; { echo FAIL; exit 1; } echo PASS '</t>
+          <t>bash -lc ' systemctl is-enabled --quiet bluetooth 2&gt;/dev/null &amp;&amp; { echo FAIL; exit 1; }; systemctl is-active --quiet bluetooth 2&gt;/dev/null &amp;&amp; { echo FAIL; exit 1; }; echo PASS '</t>
         </is>
       </c>
       <c r="H90" s="3" t="inlineStr">
@@ -5762,20 +5755,19 @@
       </c>
       <c r="J90" s="3" t="inlineStr">
         <is>
-          <t>bash: -c: line 0: syntax error near unexpected token `systemctl' | bash: -c: line 0: ` systemctl is-enabled bluetooth 2&gt;/dev/null | grep -q enabled &amp;&amp; { echo FAIL; exit 1; } systemctl is-active bluetooth 2&gt;/dev/null | grep -q active &amp;&amp; { echo FAIL; exit 1; } echo PASS '</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="K90" s="3" t="inlineStr"/>
       <c r="L90" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="M90" s="3" t="inlineStr"/>
-      <c r="N90" s="3" t="inlineStr">
-        <is>
-          <t>bash: -c: line 0: syntax error near unexpected token `systemctl'
-bash: -c: line 0: ` systemctl is-enabled bluetooth 2&gt;/dev/null | grep -q enabled &amp;&amp; { echo FAIL; exit 1; } systemctl is-active bluetooth 2&gt;/dev/null | grep -q active &amp;&amp; { echo FAIL; exit 1; } echo PASS '</t>
-        </is>
-      </c>
+      <c r="M90" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="N90" s="3" t="inlineStr"/>
       <c r="O90" s="3" t="inlineStr"/>
     </row>
     <row r="91">
@@ -6456,9 +6448,7 @@
       </c>
       <c r="G102" s="3" t="inlineStr">
         <is>
-          <t>bash -lc ' lsmod | grep -q dccp &amp;&amp; { echo FAIL; exit 1; } modprobe --showconfig | grep -Eq "dccp.*(blacklist|/bin/false)" \
-  &amp;&amp; echo PASS || echo FAIL
-'</t>
+          <t>bash -lc ' m=dccp; p=$(find /lib/modules /usr/lib/modules -type d -path "*/kernel/net/$m" 2&gt;/dev/null | head -1); [ -z "$p" ] &amp;&amp; { echo PASS; exit 0; }; lsmod | grep -qw "$m" &amp;&amp; { echo FAIL; exit 1; }; c=$(modprobe --showconfig 2&gt;/dev/null); echo "$c" | grep -Eq "^[[:space:]]*blacklist[[:space:]]+$m\b" &amp;&amp; echo "$c" | grep -Eq "^[[:space:]]*install[[:space:]]+$m[[:space:]]+/bin/(true|false)\b" &amp;&amp; echo PASS || { echo FAIL; exit 1; } '</t>
         </is>
       </c>
       <c r="H102" s="3" t="inlineStr">
@@ -6466,27 +6456,26 @@
           <t>Valida que el módulo de red DCCP no esté cargado y tenga bloqueo configurado en modprobe.</t>
         </is>
       </c>
-      <c r="I102" s="6" t="inlineStr">
-        <is>
-          <t>No cumple</t>
+      <c r="I102" s="4" t="inlineStr">
+        <is>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="J102" s="3" t="inlineStr">
         <is>
-          <t>bash: -c: line 0: syntax error near unexpected token `modprobe' | bash: -c: line 0: ` lsmod | grep -q dccp &amp;&amp; { echo FAIL; exit 1; } modprobe --showconfig | grep -Eq "dccp.*(blacklist|/bin/false)" \'</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K102" s="3" t="inlineStr"/>
       <c r="L102" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="M102" s="3" t="inlineStr"/>
-      <c r="N102" s="3" t="inlineStr">
-        <is>
-          <t>bash: -c: line 0: syntax error near unexpected token `modprobe'
-bash: -c: line 0: ` lsmod | grep -q dccp &amp;&amp; { echo FAIL; exit 1; } modprobe --showconfig | grep -Eq "dccp.*(blacklist|/bin/false)" \'</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M102" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="N102" s="3" t="inlineStr"/>
       <c r="O102" s="3" t="inlineStr"/>
     </row>
     <row r="103">
@@ -6518,9 +6507,7 @@
       </c>
       <c r="G103" s="3" t="inlineStr">
         <is>
-          <t>bash -lc ' lsmod | grep -q sctp &amp;&amp; { echo FAIL; exit 1; } modprobe --showconfig | grep -Eq "sctp.*(blacklist|/bin/false)" \
-  &amp;&amp; echo PASS || echo FAIL
-'</t>
+          <t>bash -lc ' m=sctp; p=$(find /lib/modules /usr/lib/modules -type d -path "*/kernel/net/$m" 2&gt;/dev/null | head -1); [ -z "$p" ] &amp;&amp; { echo PASS; exit 0; }; lsmod | grep -qw "$m" &amp;&amp; { echo FAIL; exit 1; }; c=$(modprobe --showconfig 2&gt;/dev/null); echo "$c" | grep -Eq "^[[:space:]]*blacklist[[:space:]]+$m\b" &amp;&amp; echo "$c" | grep -Eq "^[[:space:]]*install[[:space:]]+$m[[:space:]]+/bin/(true|false)\b" &amp;&amp; echo PASS || { echo FAIL; exit 1; } '</t>
         </is>
       </c>
       <c r="H103" s="3" t="inlineStr">
@@ -6528,27 +6515,26 @@
           <t>Valida que el módulo de red SCTP no esté cargado y tenga bloqueo configurado en modprobe.</t>
         </is>
       </c>
-      <c r="I103" s="6" t="inlineStr">
-        <is>
-          <t>No cumple</t>
+      <c r="I103" s="4" t="inlineStr">
+        <is>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="J103" s="3" t="inlineStr">
         <is>
-          <t>bash: -c: line 0: syntax error near unexpected token `modprobe' | bash: -c: line 0: ` lsmod | grep -q sctp &amp;&amp; { echo FAIL; exit 1; } modprobe --showconfig | grep -Eq "sctp.*(blacklist|/bin/false)" \'</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K103" s="3" t="inlineStr"/>
       <c r="L103" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="M103" s="3" t="inlineStr"/>
-      <c r="N103" s="3" t="inlineStr">
-        <is>
-          <t>bash: -c: line 0: syntax error near unexpected token `modprobe'
-bash: -c: line 0: ` lsmod | grep -q sctp &amp;&amp; { echo FAIL; exit 1; } modprobe --showconfig | grep -Eq "sctp.*(blacklist|/bin/false)" \'</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M103" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="N103" s="3" t="inlineStr"/>
       <c r="O103" s="3" t="inlineStr"/>
     </row>
     <row r="104">
@@ -6580,9 +6566,7 @@
       </c>
       <c r="G104" s="3" t="inlineStr">
         <is>
-          <t>bash -lc ' lsmod | grep -q rds &amp;&amp; { echo FAIL; exit 1; } modprobe --showconfig | grep -Eq "rds.*(blacklist|/bin/false)" \
-  &amp;&amp; echo PASS || echo FAIL
-'</t>
+          <t>bash -lc ' m=rds; p=$(find /lib/modules /usr/lib/modules -type d -path "*/kernel/net/$m" 2&gt;/dev/null | head -1); [ -z "$p" ] &amp;&amp; { echo PASS; exit 0; }; lsmod | grep -qw "$m" &amp;&amp; { echo FAIL; exit 1; }; c=$(modprobe --showconfig 2&gt;/dev/null); echo "$c" | grep -Eq "^[[:space:]]*blacklist[[:space:]]+$m\b" &amp;&amp; echo "$c" | grep -Eq "^[[:space:]]*install[[:space:]]+$m[[:space:]]+/bin/(true|false)\b" &amp;&amp; echo PASS || { echo FAIL; exit 1; } '</t>
         </is>
       </c>
       <c r="H104" s="3" t="inlineStr">
@@ -6597,20 +6581,19 @@
       </c>
       <c r="J104" s="3" t="inlineStr">
         <is>
-          <t>bash: -c: line 0: syntax error near unexpected token `modprobe' | bash: -c: line 0: ` lsmod | grep -q rds &amp;&amp; { echo FAIL; exit 1; } modprobe --showconfig | grep -Eq "rds.*(blacklist|/bin/false)" \'</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="K104" s="3" t="inlineStr"/>
       <c r="L104" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="M104" s="3" t="inlineStr"/>
-      <c r="N104" s="3" t="inlineStr">
-        <is>
-          <t>bash: -c: line 0: syntax error near unexpected token `modprobe'
-bash: -c: line 0: ` lsmod | grep -q rds &amp;&amp; { echo FAIL; exit 1; } modprobe --showconfig | grep -Eq "rds.*(blacklist|/bin/false)" \'</t>
-        </is>
-      </c>
+      <c r="M104" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="N104" s="3" t="inlineStr"/>
       <c r="O104" s="3" t="inlineStr"/>
     </row>
     <row r="105">
@@ -6642,9 +6625,7 @@
       </c>
       <c r="G105" s="3" t="inlineStr">
         <is>
-          <t>bash -lc ' lsmod | grep -q tipc &amp;&amp; { echo FAIL; exit 1; } modprobe --showconfig | grep -Eq "tipc.*(blacklist|/bin/false)" \
-  &amp;&amp; echo PASS || echo FAIL
-'</t>
+          <t>bash -lc ' m=tipc; p=$(find /lib/modules /usr/lib/modules -type d -path "*/kernel/net/$m" 2&gt;/dev/null | head -1); [ -z "$p" ] &amp;&amp; { echo PASS; exit 0; }; lsmod | grep -qw "$m" &amp;&amp; { echo FAIL; exit 1; }; c=$(modprobe --showconfig 2&gt;/dev/null); echo "$c" | grep -Eq "^[[:space:]]*blacklist[[:space:]]+$m\b" &amp;&amp; echo "$c" | grep -Eq "^[[:space:]]*install[[:space:]]+$m[[:space:]]+/bin/(true|false)\b" &amp;&amp; echo PASS || { echo FAIL; exit 1; } '</t>
         </is>
       </c>
       <c r="H105" s="3" t="inlineStr">
@@ -6659,20 +6640,19 @@
       </c>
       <c r="J105" s="3" t="inlineStr">
         <is>
-          <t>bash: -c: line 0: syntax error near unexpected token `modprobe' | bash: -c: line 0: ` lsmod | grep -q tipc &amp;&amp; { echo FAIL; exit 1; } modprobe --showconfig | grep -Eq "tipc.*(blacklist|/bin/false)" \'</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="K105" s="3" t="inlineStr"/>
       <c r="L105" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="M105" s="3" t="inlineStr"/>
-      <c r="N105" s="3" t="inlineStr">
-        <is>
-          <t>bash: -c: line 0: syntax error near unexpected token `modprobe'
-bash: -c: line 0: ` lsmod | grep -q tipc &amp;&amp; { echo FAIL; exit 1; } modprobe --showconfig | grep -Eq "tipc.*(blacklist|/bin/false)" \'</t>
-        </is>
-      </c>
+      <c r="M105" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="N105" s="3" t="inlineStr"/>
       <c r="O105" s="3" t="inlineStr"/>
     </row>
     <row r="106">
@@ -7953,7 +7933,7 @@
       </c>
       <c r="G127" s="3" t="inlineStr">
         <is>
-          <t>bash -lc ' grep -Ei "AllowUsers|AllowGroups|DenyUsers|DenyGroups" /etc/ssh/sshd_config /etc/ssh/sshd_config.d/* 2&gt;/dev/null \
+          <t>bash -lc ' grep -Eiq "^[[:space:]]*(AllowUsers|AllowGroups|DenyUsers|DenyGroups)[[:space:]]+" /etc/ssh/sshd_config /etc/ssh/sshd_config.d/* 2&gt;/dev/null \
   &amp;&amp; echo PASS || echo FAIL
 '</t>
         </is>
@@ -7963,14 +7943,14 @@
           <t>Valida configuración del servidor SSH para: Ensure SSH access is limited. El comando revisa /etc/ssh/sshd_config y archivos incluidos cuando aplica, retornando PASS o FAIL.</t>
         </is>
       </c>
-      <c r="I127" s="6" t="inlineStr">
-        <is>
-          <t>No cumple</t>
+      <c r="I127" s="4" t="inlineStr">
+        <is>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="J127" s="3" t="inlineStr">
         <is>
-          <t>/etc/ssh/sshd_config:AllowGroups ssh_access | FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K127" s="3" t="inlineStr"/>
@@ -7979,8 +7959,7 @@
       </c>
       <c r="M127" s="3" t="inlineStr">
         <is>
-          <t>/etc/ssh/sshd_config:AllowGroups ssh_access
-FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="N127" s="3" t="inlineStr"/>
@@ -8974,7 +8953,7 @@
       <c r="G144" s="3" t="inlineStr">
         <is>
           <t>bash -lc ' fail=0 out=""
-minlen_line=$(grep -Psi -- "^\h*minlen\h*=\h*(8|9|[1-9][0-9]+)\b" /etc/security/pwquality.conf /etc/security/pwquality.conf.d/*.conf 2&gt;/dev/null | head -n1) minclass_line=$(grep -Psi -- "^\h*minclass\h*=\h*4\b" /etc/security/pwquality.conf /etc/security/pwquality.conf.d/*.conf 2&gt;/dev/null | head -n1)
+minlen_line=$(grep -Psi -- "^[[:space:]]*minlen[[:space:]]*=[[:space:]]*(8|9|[1-9][0-9]+)\b" /etc/security/pwquality.conf /etc/security/pwquality.conf.d/*.conf 2&gt;/dev/null | head -n1) minclass_line=$(grep -Psi -- "^[[:space:]]*minclass[[:space:]]*=[[:space:]]*4\b" /etc/security/pwquality.conf /etc/security/pwquality.conf.d/*.conf 2&gt;/dev/null | head -n1)
 [ -n "$minlen_line" ] &amp;&amp; out="$out\n- minlen cumple: $minlen_line" || { out="$out\n- minlen NO cumple"; fail=1; } [ -n "$minclass_line" ] &amp;&amp; out="$out\n- minclass cumple: $minclass_line" || { out="$out\n- minclass NO cumple"; fail=1; }
 [ "$fail" -eq 0 ] &amp;&amp; echo -e "PASS$out" || { echo -e "FAIL$out"; exit 1; } '</t>
         </is>
@@ -9595,20 +9574,22 @@
       </c>
       <c r="G154" s="3" t="inlineStr">
         <is>
-          <t>bash -lc ' bad=0 mapfile -t USERS &lt; &lt;(
-  awk -F: '\''($2 !~ /^[!*]/){print $1}'\'' /etc/shadow 2&gt;/dev/null |
-  grep -Ev "^(root|tux|proactiva|iacolcoauto|ansible_test|halt|shutdown|sync|nfsnobody)$" || true
-)
-for u in "${USERS[@]}"; do
-  d=$(chage --list "$u" 2&gt;/dev/null | awk -F": " "/^Last password change/{print \$2}")
-  [ -z "$d" ] || [ "$d" = "never" ] &amp;&amp; continue
-  ts=$(date -d "$d" +%s 2&gt;/dev/null) || ts=0
-  now=$(date +%s)
-  if [ "$ts" -gt "$now" ]; then
-    echo "future:$u:$d"
+          <t>bash -lc ' EXCLUDED_RE="^(root|tux|proactiva|iacolcoauto|ansible_test|halt|shutdown|sync|nfsnobody)$" today=$(($(date +%s)/86400)) bad=0
+while IFS=: read -r user pass lastchg rest; do
+  [[ "$user" =~ $EXCLUDED_RE ]] &amp;&amp; continue
+  [[ "$pass" =~ ^[\!\*] ]] &amp;&amp; continue
+  [[ -z "$lastchg" ]] &amp;&amp; continue
+  if ! [[ "$lastchg" =~ ^[0-9]+$ ]]; then
+    echo "invalid:$user:lastchg=$lastchg"
+    bad=1
+    continue
+  fi
+  if (( lastchg &gt; today )); then
+    fecha=$(date -d "1970-01-01 UTC + $lastchg days" +%F 2&gt;/dev/null || echo "$lastchg")
+    echo "future:$user:$fecha"
     bad=1
   fi
-done
+done &lt; /etc/shadow
 [ "$bad" -eq 0 ] &amp;&amp; echo PASS || exit 1 '</t>
         </is>
       </c>
@@ -9617,26 +9598,26 @@
           <t>Recorre usuarios locales con contraseña activa, excluyendo usuarios definidos en excluded_users_regex, y valida que la fecha del último cambio de contraseña no esté en el futuro.</t>
         </is>
       </c>
-      <c r="I154" s="6" t="inlineStr">
-        <is>
-          <t>No cumple</t>
+      <c r="I154" s="4" t="inlineStr">
+        <is>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="J154" s="3" t="inlineStr">
         <is>
-          <t>bash: line 15: [: : integer expression expected</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K154" s="3" t="inlineStr"/>
       <c r="L154" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="M154" s="3" t="inlineStr"/>
-      <c r="N154" s="3" t="inlineStr">
-        <is>
-          <t>bash: line 15: [: : integer expression expected</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M154" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="N154" s="3" t="inlineStr"/>
       <c r="O154" s="3" t="inlineStr"/>
     </row>
     <row r="155">
@@ -9669,7 +9650,14 @@
       <c r="G155" s="3" t="inlineStr">
         <is>
           <t>bash -lc ' min=$(awk "/^[[:space:]]*UID_MIN[[:space:]]+/{print \$2}" /etc/login.defs) [ -z "$min" ] &amp;&amp; min=1000
-awk -F: -v min="$min" '\''($3 &lt; min &amp;&amp; $1 != "root"){print $1 ":" $7}'\'' /etc/passwd | grep -Ev "^(root|tux|proactiva|iacolcoauto|ansible_test|halt|shutdown|sync|nfsnobody):" | grep -Ev ":(/sbin/nologin|/usr/sbin/nologin|/bin/false)$" &amp;&amp; echo FAIL || echo PASS '</t>
+bad=$( awk -F: -v min="$min" '\''($3 &lt; min &amp;&amp; $1 != "root"){print $1 ":" $7}'\'' /etc/passwd | grep -Ev "^(root|tux|proactiva|iacolcoauto|ansible_test|halt|shutdown|sync|nfsnobody):" | grep -Ev ":(/sbin/nologin|/usr/sbin/nologin|/bin/nologin|/bin/false|/usr/bin/false)$" )
+if [ -n "$bad" ]; then
+  echo "$bad"
+  echo FAIL
+  exit 1
+else
+  echo PASS
+fi '</t>
         </is>
       </c>
       <c r="H155" s="3" t="inlineStr">
@@ -9677,14 +9665,14 @@
           <t>Valida que las cuentas de sistema por debajo de UID_MIN, excluyendo usuarios definidos en excluded_users_regex, tengan shell no interactiva.</t>
         </is>
       </c>
-      <c r="I155" s="6" t="inlineStr">
-        <is>
-          <t>No cumple</t>
+      <c r="I155" s="4" t="inlineStr">
+        <is>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="J155" s="3" t="inlineStr">
         <is>
-          <t>messagebus:/usr/bin/false | FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K155" s="3" t="inlineStr"/>
@@ -9693,8 +9681,7 @@
       </c>
       <c r="M155" s="3" t="inlineStr">
         <is>
-          <t>messagebus:/usr/bin/false
-FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="N155" s="3" t="inlineStr"/>
@@ -9849,7 +9836,15 @@
       </c>
       <c r="G158" s="3" t="inlineStr">
         <is>
-          <t>bash -lc ' grep -RE "^\s*TMOUT=(900|[1-8][0-9]{2}|[1-9][0-9])" /etc/profile /etc/bashrc /etc/profile.d/* 2&gt;/dev/null &amp;&amp; grep -RE "readonly TMOUT" /etc/profile /etc/bashrc /etc/profile.d/* 2&gt;/dev/null &amp;&amp; grep -RE "export TMOUT" /etc/profile /etc/bashrc /etc/profile.d/* 2&gt;/dev/null &amp;&amp; echo PASS || echo FAIL '</t>
+          <t>bash -lc ' files="/etc/profile /etc/bashrc /etc/bash.bashrc /etc/profile.d/*.sh"
+tmout_ok=$(grep -RHE "^[[:space:]]*TMOUT=([1-9][0-9]?|[1-8][0-9]{2}|900)([[:space:]]*#.*)?$" $files 2&gt;/dev/null | head -n1) readonly_ok=$(grep -RHE "^[[:space:]]*readonly[[:space:]]+TMOUT([[:space:]]*#.*)?$|^[[:space:]]*readonly[[:space:]]+TMOUT=([1-9][0-9]?|[1-8][0-9]{2}|900)([[:space:]]*#.*)?$" $files 2&gt;/dev/null | head -n1) export_ok=$(grep -RHE "^[[:space:]]*export[[:space:]]+TMOUT([[:space:]]*#.*)?$|^[[:space:]]*export[[:space:]]+TMOUT=([1-9][0-9]?|[1-8][0-9]{2}|900)([[:space:]]*#.*)?$" $files 2&gt;/dev/null | head -n1)
+[ -n "$tmout_ok" ] &amp;&amp; echo "TMOUT_OK:$tmout_ok" || echo "TMOUT_MISSING" [ -n "$readonly_ok" ] &amp;&amp; echo "READONLY_OK:$readonly_ok" || echo "READONLY_MISSING" [ -n "$export_ok" ] &amp;&amp; echo "EXPORT_OK:$export_ok" || echo "EXPORT_MISSING"
+if [ -n "$tmout_ok" ] &amp;&amp; [ -n "$readonly_ok" ] &amp;&amp; [ -n "$export_ok" ]; then
+  echo PASS
+else
+  echo FAIL
+  exit 1
+fi '</t>
         </is>
       </c>
       <c r="H158" s="3" t="inlineStr">
@@ -9857,14 +9852,14 @@
           <t>Valida que TMOUT esté configurado en 900 segundos o menos, y que además esté definido como readonly y exportado globalmente.</t>
         </is>
       </c>
-      <c r="I158" s="6" t="inlineStr">
-        <is>
-          <t>No cumple</t>
+      <c r="I158" s="4" t="inlineStr">
+        <is>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="J158" s="3" t="inlineStr">
         <is>
-          <t>/etc/profile.d/tmout.sh:TMOUT=900 | FAIL</t>
+          <t>TMOUT_OK:/etc/profile.d/tmout.sh:TMOUT=900 | READONLY_OK:/etc/profile.d/tmout.sh:readonly TMOUT | EXPORT_OK:/etc/profile.d/tmout.sh:export TMOUT | PASS</t>
         </is>
       </c>
       <c r="K158" s="3" t="inlineStr"/>
@@ -9873,8 +9868,10 @@
       </c>
       <c r="M158" s="3" t="inlineStr">
         <is>
-          <t>/etc/profile.d/tmout.sh:TMOUT=900
-FAIL</t>
+          <t>TMOUT_OK:/etc/profile.d/tmout.sh:TMOUT=900
+READONLY_OK:/etc/profile.d/tmout.sh:readonly TMOUT
+EXPORT_OK:/etc/profile.d/tmout.sh:export TMOUT
+PASS</t>
         </is>
       </c>
       <c r="N158" s="3" t="inlineStr"/>

</xml_diff>